<commit_message>
Add in Skagerak and new plots
</commit_message>
<xml_diff>
--- a/Oekokyst/Stations Nordsjøen.xlsx
+++ b/Oekokyst/Stations Nordsjøen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Dashboards\Oekokyst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{004E6BED-C829-40F0-9551-BEF66B336D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CFB1FBC-DD97-48FC-8D03-0FF8048A84F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{E969CC32-21B0-4D01-9141-475FB54071F0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{E969CC32-21B0-4D01-9141-475FB54071F0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="103">
   <si>
     <t>Stasjon</t>
   </si>
@@ -45,21 +45,12 @@
     <t>Prøvetakingsdyp</t>
   </si>
   <si>
-    <t>VT (NY_1)</t>
-  </si>
-  <si>
     <t>0, 5, 10, 20, 30</t>
   </si>
   <si>
     <t>VR49</t>
   </si>
   <si>
-    <t>VT (NY_2)</t>
-  </si>
-  <si>
-    <t>VT (NY_3)</t>
-  </si>
-  <si>
     <t>VT8</t>
   </si>
   <si>
@@ -114,12 +105,6 @@
     <t>Jøsenfjord ytre</t>
   </si>
   <si>
-    <t>Boknafjord ytre</t>
-  </si>
-  <si>
-    <t>Boknaflæet</t>
-  </si>
-  <si>
     <t>Hidlefjorden</t>
   </si>
   <si>
@@ -297,17 +282,77 @@
     <t xml:space="preserve"> m⁻¹</t>
   </si>
   <si>
-    <t>Flekkefjørd</t>
-  </si>
-  <si>
     <t>Hjelmelandsfjorden</t>
+  </si>
+  <si>
+    <t>Full_name</t>
+  </si>
+  <si>
+    <t>VT85</t>
+  </si>
+  <si>
+    <t>Prestøya</t>
+  </si>
+  <si>
+    <t>Prestøya (VT85)</t>
+  </si>
+  <si>
+    <t>02.01-128017</t>
+  </si>
+  <si>
+    <t>Jøsenfjord ytre (VR49)</t>
+  </si>
+  <si>
+    <t>VR62</t>
+  </si>
+  <si>
+    <t>Båtholmen</t>
+  </si>
+  <si>
+    <t>Båtholmen (VR62)</t>
+  </si>
+  <si>
+    <t>02.42-128015</t>
+  </si>
+  <si>
+    <t>VR63</t>
+  </si>
+  <si>
+    <t>Brattholmen</t>
+  </si>
+  <si>
+    <t>Brattholmen (VR63)</t>
+  </si>
+  <si>
+    <t>02.42-128016</t>
+  </si>
+  <si>
+    <t>Hidlefjorden (VT8)</t>
+  </si>
+  <si>
+    <t>Hjelmelandsfjorden (VT83)</t>
+  </si>
+  <si>
+    <t>Bjørnafjorden (VT70)</t>
+  </si>
+  <si>
+    <t>Maurangsfjorden (VT74)</t>
+  </si>
+  <si>
+    <t>Tveitneset (VT53)</t>
+  </si>
+  <si>
+    <t>Kykjebø (VT16)</t>
+  </si>
+  <si>
+    <t>Nærnes (VT79)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -323,29 +368,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -353,71 +385,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -757,7 +731,7 @@
   <cols>
     <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -765,283 +739,301 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2">
+        <v>240.4365</v>
+      </c>
+      <c r="G2">
+        <v>6484606.2429999998</v>
+      </c>
+      <c r="H2">
+        <v>6.4794442999999999</v>
+      </c>
+      <c r="I2">
+        <v>58.217515499999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3">
+        <v>1909.6070999999999</v>
+      </c>
+      <c r="G3">
+        <v>6603444.8770000003</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4">
+        <v>-55637.842799999999</v>
+      </c>
+      <c r="G4">
+        <v>6586705.6500000004</v>
+      </c>
+      <c r="H4">
+        <v>5.2912017000000002</v>
+      </c>
+      <c r="I4">
+        <v>59.055045700000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5">
+        <v>-44280.765899999999</v>
+      </c>
+      <c r="G5">
+        <v>6609311.4720000001</v>
+      </c>
+      <c r="H5">
+        <v>5.4301725000000003</v>
+      </c>
+      <c r="I5">
+        <v>59.269851600000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6">
+        <v>-26463.599999999999</v>
+      </c>
+      <c r="G6">
+        <v>6583850.7999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7">
+        <v>-4774.7</v>
+      </c>
+      <c r="G7">
+        <v>6600828.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="C8" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2">
-        <v>240.4365</v>
-      </c>
-      <c r="F2">
-        <v>6484606.2429</v>
-      </c>
-      <c r="G2" s="5">
-        <v>6.4794442999999999</v>
-      </c>
-      <c r="H2" s="5">
-        <v>58.217515499999998</v>
-      </c>
-      <c r="I2" s="5"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="5" t="s">
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8">
+        <v>-28419.4</v>
+      </c>
+      <c r="G8">
+        <v>6701234.7999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>24</v>
       </c>
-      <c r="C3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3">
-        <v>1909.60709999967</v>
-      </c>
-      <c r="F3">
-        <v>6603444.8770000003</v>
-      </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="7" t="s">
+      <c r="C9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9">
+        <v>9942.7999999999993</v>
+      </c>
+      <c r="G9">
+        <v>6696066</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
         <v>25</v>
       </c>
-      <c r="C4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4">
-        <v>-55637.842799999999</v>
-      </c>
-      <c r="F4">
-        <v>6586705.6496000001</v>
-      </c>
-      <c r="G4" s="5">
-        <v>5.2912017000000002</v>
-      </c>
-      <c r="H4" s="5">
-        <v>59.055045700000001</v>
-      </c>
-      <c r="I4" s="5"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="7" t="s">
+      <c r="C10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10">
+        <v>29230.400000000001</v>
+      </c>
+      <c r="G10">
+        <v>6726778.7999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="C5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5">
-        <v>-44280.765899999999</v>
-      </c>
-      <c r="F5">
-        <v>6609311.4721999997</v>
-      </c>
-      <c r="G5" s="5">
-        <v>5.4301725000000003</v>
-      </c>
-      <c r="H5" s="5">
-        <v>59.269851600000003</v>
-      </c>
-      <c r="I5" s="5"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="C11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11">
+        <v>14003.4</v>
+      </c>
+      <c r="G11">
+        <v>6812759.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>-26463.599999999598</v>
-      </c>
-      <c r="F6">
-        <v>6583850.7999999998</v>
-      </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" t="s">
-        <v>3</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7">
-        <v>-4774.7000000001799</v>
-      </c>
-      <c r="F7">
-        <v>6600828.5</v>
-      </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8">
-        <v>-28419.4000000003</v>
-      </c>
-      <c r="F8">
-        <v>6701234.7999999998</v>
-      </c>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" t="s">
-        <v>3</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
         <v>18</v>
       </c>
-      <c r="E9">
-        <v>9942.7999999998101</v>
-      </c>
-      <c r="F9">
-        <v>6696066</v>
-      </c>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10">
-        <v>29230.4000000003</v>
-      </c>
-      <c r="F10">
-        <v>6726778.7999999998</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E11">
-        <v>14003.4000000003</v>
-      </c>
-      <c r="F11">
-        <v>6812759.5</v>
-      </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12">
-        <v>71014.9000000003</v>
-      </c>
       <c r="F12">
+        <v>71014.899999999994</v>
+      </c>
+      <c r="G12">
         <v>6788449.2999999998</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1058,225 +1050,231 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
         <v>53</v>
-      </c>
-      <c r="B20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" t="s">
-        <v>58</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{85110470-9488-4156-833d-c297ee816837}" enabled="1" method="Privileged" siteId="{ce25ca93-004f-44f4-a6b5-eb22b45815aa}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>